<commit_message>
Implement Excel outputs, add parameters to data product links
Extensive documentation improvements.
</commit_message>
<xml_diff>
--- a/catalog.xlsx
+++ b/catalog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="103">
   <si>
     <t>TileID</t>
   </si>
@@ -223,16 +223,103 @@
     <t>annually</t>
   </si>
   <si>
-    <t>https://www.arcgis.com/apps/dashboards/025b75f3490b4e79ae764e2c27c09a06</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/d1bb7ef5468f495788703352b1c5f896</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/2d3cc0a173d949f0a1a39146b37e1831</t>
-  </si>
-  <si>
-    <t>https://morpc1-my.sharepoint.com/:w:/g/personal/aporr_morpc_org/EdF9OgInIZdOk9Sz3aJSVT8BPvXp4N495QUN2PvK5NBBjQ?e=b30KGA</t>
+    <t>https://www.arcgis.com/apps/dashboards/025b75f3490b4e79ae764e2c27c09a06#geoName=Delaware County</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/025b75f3490b4e79ae764e2c27c09a06#geoName=Fairfield County</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/025b75f3490b4e79ae764e2c27c09a06#geoName=Franklin County</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/025b75f3490b4e79ae764e2c27c09a06#geoName=Knox County</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/025b75f3490b4e79ae764e2c27c09a06#geoName=Licking County</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/025b75f3490b4e79ae764e2c27c09a06#geoName=Madison County</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/025b75f3490b4e79ae764e2c27c09a06#geoName=Marion County</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/025b75f3490b4e79ae764e2c27c09a06#geoName=Morrow County</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/025b75f3490b4e79ae764e2c27c09a06#geoName=Pickaway County</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/025b75f3490b4e79ae764e2c27c09a06#geoName=Union County</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/025b75f3490b4e79ae764e2c27c09a06#geoName=10-County Region</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/d1bb7ef5468f495788703352b1c5f896#geoName=Delaware County</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/d1bb7ef5468f495788703352b1c5f896#geoName=Fairfield County</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/d1bb7ef5468f495788703352b1c5f896#geoName=Franklin County</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/d1bb7ef5468f495788703352b1c5f896#geoName=Knox County</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/d1bb7ef5468f495788703352b1c5f896#geoName=Licking County</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/d1bb7ef5468f495788703352b1c5f896#geoName=Madison County</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/d1bb7ef5468f495788703352b1c5f896#geoName=Marion County</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/d1bb7ef5468f495788703352b1c5f896#geoName=Morrow County</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/d1bb7ef5468f495788703352b1c5f896#geoName=Pickaway County</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/d1bb7ef5468f495788703352b1c5f896#geoName=Union County</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/d1bb7ef5468f495788703352b1c5f896#geoName=10-County Region</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/2d3cc0a173d949f0a1a39146b37e1831#geoName=Delaware County</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/2d3cc0a173d949f0a1a39146b37e1831#geoName=Fairfield County</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/2d3cc0a173d949f0a1a39146b37e1831#geoName=Franklin County</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/2d3cc0a173d949f0a1a39146b37e1831#geoName=Knox County</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/2d3cc0a173d949f0a1a39146b37e1831#geoName=Licking County</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/2d3cc0a173d949f0a1a39146b37e1831#geoName=Madison County</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/2d3cc0a173d949f0a1a39146b37e1831#geoName=Marion County</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/2d3cc0a173d949f0a1a39146b37e1831#geoName=Morrow County</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/2d3cc0a173d949f0a1a39146b37e1831#geoName=Pickaway County</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/2d3cc0a173d949f0a1a39146b37e1831#geoName=Union County</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/2d3cc0a173d949f0a1a39146b37e1831#geoName=10-County Region</t>
   </si>
   <si>
     <t>https://github.com/morpc-insights/insights-crashes</t>
@@ -690,11 +777,8 @@
       <c r="N2" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="O2" s="2" t="s">
-        <v>72</v>
-      </c>
       <c r="P2" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3" spans="1:16">
@@ -726,13 +810,10 @@
         <v>68</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="O3" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" spans="1:16">
@@ -764,13 +845,10 @@
         <v>68</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="O4" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="P4" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="5" spans="1:16">
@@ -802,13 +880,10 @@
         <v>68</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="O5" s="2" t="s">
         <v>72</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="6" spans="1:16">
@@ -840,13 +915,10 @@
         <v>68</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="O6" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="P6" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="7" spans="1:16">
@@ -878,13 +950,10 @@
         <v>68</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="O7" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="P7" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="8" spans="1:16">
@@ -916,13 +985,10 @@
         <v>68</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="O8" s="2" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="P8" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="9" spans="1:16">
@@ -954,13 +1020,10 @@
         <v>68</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="O9" s="2" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="P9" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="10" spans="1:16">
@@ -992,13 +1055,10 @@
         <v>68</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="O10" s="2" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="P10" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="11" spans="1:16">
@@ -1030,13 +1090,10 @@
         <v>68</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="O11" s="2" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="P11" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="12" spans="1:16">
@@ -1068,13 +1125,10 @@
         <v>68</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="O12" s="2" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="P12" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="13" spans="1:16">
@@ -1106,13 +1160,10 @@
         <v>68</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="O13" s="2" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="P13" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="14" spans="1:16">
@@ -1144,13 +1195,10 @@
         <v>68</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="O14" s="2" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="P14" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="15" spans="1:16">
@@ -1182,13 +1230,10 @@
         <v>68</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="O15" s="2" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="P15" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="16" spans="1:16">
@@ -1220,13 +1265,10 @@
         <v>68</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="O16" s="2" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="P16" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="17" spans="2:16">
@@ -1258,13 +1300,10 @@
         <v>68</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="O17" s="2" t="s">
-        <v>72</v>
+        <v>84</v>
       </c>
       <c r="P17" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="18" spans="2:16">
@@ -1296,13 +1335,10 @@
         <v>68</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="O18" s="2" t="s">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="P18" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="19" spans="2:16">
@@ -1334,13 +1370,10 @@
         <v>68</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="O19" s="2" t="s">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="P19" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="20" spans="2:16">
@@ -1372,13 +1405,10 @@
         <v>68</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="O20" s="2" t="s">
-        <v>72</v>
+        <v>87</v>
       </c>
       <c r="P20" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="21" spans="2:16">
@@ -1410,13 +1440,10 @@
         <v>68</v>
       </c>
       <c r="N21" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="O21" s="2" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="P21" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="22" spans="2:16">
@@ -1448,13 +1475,10 @@
         <v>68</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="O22" s="2" t="s">
-        <v>72</v>
+        <v>89</v>
       </c>
       <c r="P22" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="23" spans="2:16">
@@ -1486,13 +1510,10 @@
         <v>68</v>
       </c>
       <c r="N23" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="O23" s="2" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="P23" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="24" spans="2:16">
@@ -1524,13 +1545,10 @@
         <v>68</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="O24" s="2" t="s">
-        <v>72</v>
+        <v>91</v>
       </c>
       <c r="P24" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="25" spans="2:16">
@@ -1562,13 +1580,10 @@
         <v>68</v>
       </c>
       <c r="N25" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="O25" s="2" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="P25" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="26" spans="2:16">
@@ -1600,13 +1615,10 @@
         <v>68</v>
       </c>
       <c r="N26" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="O26" s="2" t="s">
-        <v>72</v>
+        <v>93</v>
       </c>
       <c r="P26" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="27" spans="2:16">
@@ -1638,13 +1650,10 @@
         <v>68</v>
       </c>
       <c r="N27" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="O27" s="2" t="s">
-        <v>72</v>
+        <v>94</v>
       </c>
       <c r="P27" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="28" spans="2:16">
@@ -1676,13 +1685,10 @@
         <v>68</v>
       </c>
       <c r="N28" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="O28" s="2" t="s">
-        <v>72</v>
+        <v>95</v>
       </c>
       <c r="P28" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="29" spans="2:16">
@@ -1714,13 +1720,10 @@
         <v>68</v>
       </c>
       <c r="N29" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="O29" s="2" t="s">
-        <v>72</v>
+        <v>96</v>
       </c>
       <c r="P29" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="30" spans="2:16">
@@ -1752,13 +1755,10 @@
         <v>68</v>
       </c>
       <c r="N30" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="O30" s="2" t="s">
-        <v>72</v>
+        <v>97</v>
       </c>
       <c r="P30" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="31" spans="2:16">
@@ -1790,13 +1790,10 @@
         <v>68</v>
       </c>
       <c r="N31" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="O31" s="2" t="s">
-        <v>72</v>
+        <v>98</v>
       </c>
       <c r="P31" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="32" spans="2:16">
@@ -1828,13 +1825,10 @@
         <v>68</v>
       </c>
       <c r="N32" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="O32" s="2" t="s">
-        <v>72</v>
+        <v>99</v>
       </c>
       <c r="P32" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="33" spans="2:16">
@@ -1866,13 +1860,10 @@
         <v>68</v>
       </c>
       <c r="N33" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="O33" s="2" t="s">
-        <v>72</v>
+        <v>100</v>
       </c>
       <c r="P33" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="34" spans="2:16">
@@ -1904,149 +1895,113 @@
         <v>68</v>
       </c>
       <c r="N34" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="O34" s="2" t="s">
-        <v>72</v>
+        <v>101</v>
       </c>
       <c r="P34" s="2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="I2" r:id="rId1"/>
-    <hyperlink ref="N2" r:id="rId2"/>
-    <hyperlink ref="O2" r:id="rId3"/>
-    <hyperlink ref="P2" r:id="rId4"/>
-    <hyperlink ref="I3" r:id="rId5"/>
-    <hyperlink ref="N3" r:id="rId6"/>
-    <hyperlink ref="O3" r:id="rId7"/>
-    <hyperlink ref="P3" r:id="rId8"/>
-    <hyperlink ref="I4" r:id="rId9"/>
-    <hyperlink ref="N4" r:id="rId10"/>
-    <hyperlink ref="O4" r:id="rId11"/>
-    <hyperlink ref="P4" r:id="rId12"/>
-    <hyperlink ref="I5" r:id="rId13"/>
-    <hyperlink ref="N5" r:id="rId14"/>
-    <hyperlink ref="O5" r:id="rId15"/>
-    <hyperlink ref="P5" r:id="rId16"/>
-    <hyperlink ref="I6" r:id="rId17"/>
-    <hyperlink ref="N6" r:id="rId18"/>
-    <hyperlink ref="O6" r:id="rId19"/>
-    <hyperlink ref="P6" r:id="rId20"/>
-    <hyperlink ref="I7" r:id="rId21"/>
-    <hyperlink ref="N7" r:id="rId22"/>
-    <hyperlink ref="O7" r:id="rId23"/>
-    <hyperlink ref="P7" r:id="rId24"/>
-    <hyperlink ref="I8" r:id="rId25"/>
-    <hyperlink ref="N8" r:id="rId26"/>
-    <hyperlink ref="O8" r:id="rId27"/>
-    <hyperlink ref="P8" r:id="rId28"/>
-    <hyperlink ref="I9" r:id="rId29"/>
-    <hyperlink ref="N9" r:id="rId30"/>
-    <hyperlink ref="O9" r:id="rId31"/>
-    <hyperlink ref="P9" r:id="rId32"/>
-    <hyperlink ref="I10" r:id="rId33"/>
-    <hyperlink ref="N10" r:id="rId34"/>
-    <hyperlink ref="O10" r:id="rId35"/>
-    <hyperlink ref="P10" r:id="rId36"/>
-    <hyperlink ref="I11" r:id="rId37"/>
-    <hyperlink ref="N11" r:id="rId38"/>
-    <hyperlink ref="O11" r:id="rId39"/>
-    <hyperlink ref="P11" r:id="rId40"/>
-    <hyperlink ref="I12" r:id="rId41"/>
-    <hyperlink ref="N12" r:id="rId42"/>
-    <hyperlink ref="O12" r:id="rId43"/>
-    <hyperlink ref="P12" r:id="rId44"/>
-    <hyperlink ref="I13" r:id="rId45"/>
-    <hyperlink ref="N13" r:id="rId46"/>
-    <hyperlink ref="O13" r:id="rId47"/>
-    <hyperlink ref="P13" r:id="rId48"/>
-    <hyperlink ref="I14" r:id="rId49"/>
-    <hyperlink ref="N14" r:id="rId50"/>
-    <hyperlink ref="O14" r:id="rId51"/>
-    <hyperlink ref="P14" r:id="rId52"/>
-    <hyperlink ref="I15" r:id="rId53"/>
-    <hyperlink ref="N15" r:id="rId54"/>
-    <hyperlink ref="O15" r:id="rId55"/>
-    <hyperlink ref="P15" r:id="rId56"/>
-    <hyperlink ref="I16" r:id="rId57"/>
-    <hyperlink ref="N16" r:id="rId58"/>
-    <hyperlink ref="O16" r:id="rId59"/>
-    <hyperlink ref="P16" r:id="rId60"/>
-    <hyperlink ref="I17" r:id="rId61"/>
-    <hyperlink ref="N17" r:id="rId62"/>
-    <hyperlink ref="O17" r:id="rId63"/>
-    <hyperlink ref="P17" r:id="rId64"/>
-    <hyperlink ref="I18" r:id="rId65"/>
-    <hyperlink ref="N18" r:id="rId66"/>
-    <hyperlink ref="O18" r:id="rId67"/>
-    <hyperlink ref="P18" r:id="rId68"/>
-    <hyperlink ref="I19" r:id="rId69"/>
-    <hyperlink ref="N19" r:id="rId70"/>
-    <hyperlink ref="O19" r:id="rId71"/>
-    <hyperlink ref="P19" r:id="rId72"/>
-    <hyperlink ref="I20" r:id="rId73"/>
-    <hyperlink ref="N20" r:id="rId74"/>
-    <hyperlink ref="O20" r:id="rId75"/>
-    <hyperlink ref="P20" r:id="rId76"/>
-    <hyperlink ref="I21" r:id="rId77"/>
-    <hyperlink ref="N21" r:id="rId78"/>
-    <hyperlink ref="O21" r:id="rId79"/>
-    <hyperlink ref="P21" r:id="rId80"/>
-    <hyperlink ref="I22" r:id="rId81"/>
-    <hyperlink ref="N22" r:id="rId82"/>
-    <hyperlink ref="O22" r:id="rId83"/>
-    <hyperlink ref="P22" r:id="rId84"/>
-    <hyperlink ref="I23" r:id="rId85"/>
-    <hyperlink ref="N23" r:id="rId86"/>
-    <hyperlink ref="O23" r:id="rId87"/>
-    <hyperlink ref="P23" r:id="rId88"/>
-    <hyperlink ref="I24" r:id="rId89"/>
-    <hyperlink ref="N24" r:id="rId90"/>
-    <hyperlink ref="O24" r:id="rId91"/>
-    <hyperlink ref="P24" r:id="rId92"/>
-    <hyperlink ref="I25" r:id="rId93"/>
-    <hyperlink ref="N25" r:id="rId94"/>
-    <hyperlink ref="O25" r:id="rId95"/>
-    <hyperlink ref="P25" r:id="rId96"/>
-    <hyperlink ref="I26" r:id="rId97"/>
-    <hyperlink ref="N26" r:id="rId98"/>
-    <hyperlink ref="O26" r:id="rId99"/>
-    <hyperlink ref="P26" r:id="rId100"/>
-    <hyperlink ref="I27" r:id="rId101"/>
-    <hyperlink ref="N27" r:id="rId102"/>
-    <hyperlink ref="O27" r:id="rId103"/>
-    <hyperlink ref="P27" r:id="rId104"/>
-    <hyperlink ref="I28" r:id="rId105"/>
-    <hyperlink ref="N28" r:id="rId106"/>
-    <hyperlink ref="O28" r:id="rId107"/>
-    <hyperlink ref="P28" r:id="rId108"/>
-    <hyperlink ref="I29" r:id="rId109"/>
-    <hyperlink ref="N29" r:id="rId110"/>
-    <hyperlink ref="O29" r:id="rId111"/>
-    <hyperlink ref="P29" r:id="rId112"/>
-    <hyperlink ref="I30" r:id="rId113"/>
-    <hyperlink ref="N30" r:id="rId114"/>
-    <hyperlink ref="O30" r:id="rId115"/>
-    <hyperlink ref="P30" r:id="rId116"/>
-    <hyperlink ref="I31" r:id="rId117"/>
-    <hyperlink ref="N31" r:id="rId118"/>
-    <hyperlink ref="O31" r:id="rId119"/>
-    <hyperlink ref="P31" r:id="rId120"/>
-    <hyperlink ref="I32" r:id="rId121"/>
-    <hyperlink ref="N32" r:id="rId122"/>
-    <hyperlink ref="O32" r:id="rId123"/>
-    <hyperlink ref="P32" r:id="rId124"/>
-    <hyperlink ref="I33" r:id="rId125"/>
-    <hyperlink ref="N33" r:id="rId126"/>
-    <hyperlink ref="O33" r:id="rId127"/>
-    <hyperlink ref="P33" r:id="rId128"/>
-    <hyperlink ref="I34" r:id="rId129"/>
-    <hyperlink ref="N34" r:id="rId130"/>
-    <hyperlink ref="O34" r:id="rId131"/>
-    <hyperlink ref="P34" r:id="rId132"/>
+    <hyperlink ref="N2" r:id="rId2" location="geoName=Delaware County"/>
+    <hyperlink ref="P2" r:id="rId3"/>
+    <hyperlink ref="I3" r:id="rId4"/>
+    <hyperlink ref="N3" r:id="rId5" location="geoName=Fairfield County"/>
+    <hyperlink ref="P3" r:id="rId6"/>
+    <hyperlink ref="I4" r:id="rId7"/>
+    <hyperlink ref="N4" r:id="rId8" location="geoName=Franklin County"/>
+    <hyperlink ref="P4" r:id="rId9"/>
+    <hyperlink ref="I5" r:id="rId10"/>
+    <hyperlink ref="N5" r:id="rId11" location="geoName=Knox County"/>
+    <hyperlink ref="P5" r:id="rId12"/>
+    <hyperlink ref="I6" r:id="rId13"/>
+    <hyperlink ref="N6" r:id="rId14" location="geoName=Licking County"/>
+    <hyperlink ref="P6" r:id="rId15"/>
+    <hyperlink ref="I7" r:id="rId16"/>
+    <hyperlink ref="N7" r:id="rId17" location="geoName=Madison County"/>
+    <hyperlink ref="P7" r:id="rId18"/>
+    <hyperlink ref="I8" r:id="rId19"/>
+    <hyperlink ref="N8" r:id="rId20" location="geoName=Marion County"/>
+    <hyperlink ref="P8" r:id="rId21"/>
+    <hyperlink ref="I9" r:id="rId22"/>
+    <hyperlink ref="N9" r:id="rId23" location="geoName=Morrow County"/>
+    <hyperlink ref="P9" r:id="rId24"/>
+    <hyperlink ref="I10" r:id="rId25"/>
+    <hyperlink ref="N10" r:id="rId26" location="geoName=Pickaway County"/>
+    <hyperlink ref="P10" r:id="rId27"/>
+    <hyperlink ref="I11" r:id="rId28"/>
+    <hyperlink ref="N11" r:id="rId29" location="geoName=Union County"/>
+    <hyperlink ref="P11" r:id="rId30"/>
+    <hyperlink ref="I12" r:id="rId31"/>
+    <hyperlink ref="N12" r:id="rId32" location="geoName=10-County Region"/>
+    <hyperlink ref="P12" r:id="rId33"/>
+    <hyperlink ref="I13" r:id="rId34"/>
+    <hyperlink ref="N13" r:id="rId35" location="geoName=Delaware County"/>
+    <hyperlink ref="P13" r:id="rId36"/>
+    <hyperlink ref="I14" r:id="rId37"/>
+    <hyperlink ref="N14" r:id="rId38" location="geoName=Fairfield County"/>
+    <hyperlink ref="P14" r:id="rId39"/>
+    <hyperlink ref="I15" r:id="rId40"/>
+    <hyperlink ref="N15" r:id="rId41" location="geoName=Franklin County"/>
+    <hyperlink ref="P15" r:id="rId42"/>
+    <hyperlink ref="I16" r:id="rId43"/>
+    <hyperlink ref="N16" r:id="rId44" location="geoName=Knox County"/>
+    <hyperlink ref="P16" r:id="rId45"/>
+    <hyperlink ref="I17" r:id="rId46"/>
+    <hyperlink ref="N17" r:id="rId47" location="geoName=Licking County"/>
+    <hyperlink ref="P17" r:id="rId48"/>
+    <hyperlink ref="I18" r:id="rId49"/>
+    <hyperlink ref="N18" r:id="rId50" location="geoName=Madison County"/>
+    <hyperlink ref="P18" r:id="rId51"/>
+    <hyperlink ref="I19" r:id="rId52"/>
+    <hyperlink ref="N19" r:id="rId53" location="geoName=Marion County"/>
+    <hyperlink ref="P19" r:id="rId54"/>
+    <hyperlink ref="I20" r:id="rId55"/>
+    <hyperlink ref="N20" r:id="rId56" location="geoName=Morrow County"/>
+    <hyperlink ref="P20" r:id="rId57"/>
+    <hyperlink ref="I21" r:id="rId58"/>
+    <hyperlink ref="N21" r:id="rId59" location="geoName=Pickaway County"/>
+    <hyperlink ref="P21" r:id="rId60"/>
+    <hyperlink ref="I22" r:id="rId61"/>
+    <hyperlink ref="N22" r:id="rId62" location="geoName=Union County"/>
+    <hyperlink ref="P22" r:id="rId63"/>
+    <hyperlink ref="I23" r:id="rId64"/>
+    <hyperlink ref="N23" r:id="rId65" location="geoName=10-County Region"/>
+    <hyperlink ref="P23" r:id="rId66"/>
+    <hyperlink ref="I24" r:id="rId67"/>
+    <hyperlink ref="N24" r:id="rId68" location="geoName=Delaware County"/>
+    <hyperlink ref="P24" r:id="rId69"/>
+    <hyperlink ref="I25" r:id="rId70"/>
+    <hyperlink ref="N25" r:id="rId71" location="geoName=Fairfield County"/>
+    <hyperlink ref="P25" r:id="rId72"/>
+    <hyperlink ref="I26" r:id="rId73"/>
+    <hyperlink ref="N26" r:id="rId74" location="geoName=Franklin County"/>
+    <hyperlink ref="P26" r:id="rId75"/>
+    <hyperlink ref="I27" r:id="rId76"/>
+    <hyperlink ref="N27" r:id="rId77" location="geoName=Knox County"/>
+    <hyperlink ref="P27" r:id="rId78"/>
+    <hyperlink ref="I28" r:id="rId79"/>
+    <hyperlink ref="N28" r:id="rId80" location="geoName=Licking County"/>
+    <hyperlink ref="P28" r:id="rId81"/>
+    <hyperlink ref="I29" r:id="rId82"/>
+    <hyperlink ref="N29" r:id="rId83" location="geoName=Madison County"/>
+    <hyperlink ref="P29" r:id="rId84"/>
+    <hyperlink ref="I30" r:id="rId85"/>
+    <hyperlink ref="N30" r:id="rId86" location="geoName=Marion County"/>
+    <hyperlink ref="P30" r:id="rId87"/>
+    <hyperlink ref="I31" r:id="rId88"/>
+    <hyperlink ref="N31" r:id="rId89" location="geoName=Morrow County"/>
+    <hyperlink ref="P31" r:id="rId90"/>
+    <hyperlink ref="I32" r:id="rId91"/>
+    <hyperlink ref="N32" r:id="rId92" location="geoName=Pickaway County"/>
+    <hyperlink ref="P32" r:id="rId93"/>
+    <hyperlink ref="I33" r:id="rId94"/>
+    <hyperlink ref="N33" r:id="rId95" location="geoName=Union County"/>
+    <hyperlink ref="P33" r:id="rId96"/>
+    <hyperlink ref="I34" r:id="rId97"/>
+    <hyperlink ref="N34" r:id="rId98" location="geoName=10-County Region"/>
+    <hyperlink ref="P34" r:id="rId99"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>